<commit_message>
closeout report is done in mars
</commit_message>
<xml_diff>
--- a/007_Can_SapAriba_Mars_Performer/Data/SapAribaMarsPerformerConfig.xlsx
+++ b/007_Can_SapAriba_Mars_Performer/Data/SapAribaMarsPerformerConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\1files\uipath\projects\007_Can_SapAriba_Mars\007_Can_SapAriba_Mars_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E405EA0-51DF-40EB-84E5-E9B238C4973C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA01E976-2B02-4236-8813-504B7907D2C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13935" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="84">
   <si>
     <t>Name</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>bulent.yarbasi@linktera.com</t>
+  </si>
+  <si>
+    <t>outputFolderPath</t>
+  </si>
+  <si>
+    <t>C:\1files\uipath\can_ar_ariba\mars\invoice_reports\</t>
   </si>
 </sst>
 </file>
@@ -800,7 +806,14 @@
     <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" t="s">
+        <v>83</v>
+      </c>
+    </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>